<commit_message>
just some file adjustment
</commit_message>
<xml_diff>
--- a/tests/test_data/spectro_files/meas_hpge_calib.xlsx
+++ b/tests/test_data/spectro_files/meas_hpge_calib.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\ZPyDosi\zpydosi\tests\test_data\spectro_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83F54D-A0EA-41E9-A30F-E398B89378E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9E0D73-2728-40FD-A8DE-00E83540E760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -153,9 +153,6 @@
     <t xml:space="preserve">1st time with a material: </t>
   </si>
   <si>
-    <t>python3   $petale_analysis/python/hpge/spectrum_calib2.py        csv=$path_csv   case=L1_p13_mai_2020</t>
-  </si>
-  <si>
     <t>############################################################### DATA</t>
   </si>
   <si>
@@ -447,9 +444,6 @@
     <t>1st time with HPGe</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_nrj1.py           tka=data/todo.TKA</t>
-  </si>
-  <si>
     <t>labo_ref</t>
   </si>
   <si>
@@ -462,9 +456,6 @@
     <t>1st time with material</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_plot4.py         csv=$path_csv   case=todo</t>
-  </si>
-  <si>
     <t>path_bkg</t>
   </si>
   <si>
@@ -474,9 +465,6 @@
     <t>for each measurement</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=todo  serv=1 </t>
-  </si>
-  <si>
     <t>data/yy_mm_dd_hh_mm_ss_hpge_position_material_blabla.TKA</t>
   </si>
   <si>
@@ -492,18 +480,12 @@
     <t>##############################################################</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_nrj1.py            tka=../irrad/petale/hpge_data/calib/Fu/2020_09_29_12_00_00_Fu_p13_Eu152-2020.TKA</t>
-  </si>
-  <si>
     <t>############################## Fu #############################</t>
   </si>
   <si>
     <t>############################################################### Eu 152</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_plot4.py         csv=$path_csv   case=Eu152_Fu</t>
-  </si>
-  <si>
     <t>Eu152_Fu</t>
   </si>
   <si>
@@ -528,9 +510,6 @@
     <t>Co60_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Co60_Fu   serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_01_12_00_00_Fu_p13_24h_Co60-2020.TKA</t>
   </si>
   <si>
@@ -540,9 +519,6 @@
     <t>Mn54_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Mn54_Fu   serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_02_12_00_00_Fe_p13_Mn54-2020.TKA</t>
   </si>
   <si>
@@ -552,9 +528,6 @@
     <t>Cs137_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Cs137_Fu    serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_02_12_00_00_Fu_p13_Cs137-2020.TKA</t>
   </si>
   <si>
@@ -564,9 +537,6 @@
     <t>Cs134_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Cs134_Fu    serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_06_12_00_00_Fu_p13_Cs134-2020.TKA</t>
   </si>
   <si>
@@ -576,9 +546,6 @@
     <t>Zn65_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Zn65_Fu     serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_06_12_00_00_Fu_p13_Zn65-2020.TKA</t>
   </si>
   <si>
@@ -588,9 +555,6 @@
     <t>Co57_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Co57_Fu    serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_05_12_00_00_Fu_p13_Co57-2020.TKA</t>
   </si>
   <si>
@@ -600,9 +564,6 @@
     <t>Na22_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Na22_Fu   serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_10_01_12_00_00_Fu_p13_Na22-2020.TKA</t>
   </si>
   <si>
@@ -612,9 +573,6 @@
     <t>Ba133_Fu</t>
   </si>
   <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Ba133_Fu    serv=1 </t>
-  </si>
-  <si>
     <t>../irrad/petale/hpge_data/calib/Fu/2020_09_30_12_00_00_Fu_p13_Ba133-2020.TKA</t>
   </si>
   <si>
@@ -624,15 +582,9 @@
     <t>Fu_p13_oct_2020</t>
   </si>
   <si>
-    <t>python3   $petale_analysis/python/hpge/check_cascade1.py</t>
-  </si>
-  <si>
     <t>fit_order</t>
   </si>
   <si>
-    <t>python3   $petale_analysis/python/hpge/spectrum_calib2.py   csv=$path_csv   case=Fu_p13_oct_2020</t>
-  </si>
-  <si>
     <t>sigma_cut [%]</t>
   </si>
   <si>
@@ -660,28 +612,76 @@
     <t>spectrum_calib.py</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_nrj2.py            tka=data/2020_05_29_13_55_26_L1_p13_200h_Eu152-2020.TKA</t>
-  </si>
-  <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_counter11.py   csv=$path_csv   case=Eu152_L1_p13_mai2020</t>
-  </si>
-  <si>
     <t>test_data/spectro_files/background_spectra/2020_10_19_12_00_00_Fu_90h_bkg.TKA</t>
   </si>
   <si>
     <t>test_data/spectro_files/calib_spectra/2020_09_29_12_00_00_Fu_p13_Eu152-2020.TKA</t>
   </si>
   <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_nrj2.py            tka=test_data/spectro_files/calib_spectra/2020_09_29_12_00_00_Fu_p13_Eu152-2020.TKA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter11.py  csv=$path_csv   case=Eu152_Fu  serv=1 </t>
-  </si>
-  <si>
-    <t>python3  $petale_analysis/python/hpge/spectrum_plot4.py         csv=$path_csv   case=Eu152-2021_Fu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python3  $petale_analysis/python/hpge/spectrum_counter5.py  csv=$path_csv   case=Eu152-2021_Fu  serv=1 </t>
+    <t>python3 spectrum_nrj2.py            tka=data/2020_05_29_13_55_26_L1_p13_200h_Eu152-2020.TKA</t>
+  </si>
+  <si>
+    <t>python3 spectrum_counter11.py   csv=$path_csv   case=Eu152_L1_p13_mai2020</t>
+  </si>
+  <si>
+    <t>python3  spectrum_calib2.py        csv=$path_csv   case=L1_p13_mai_2020</t>
+  </si>
+  <si>
+    <t>python3 spectrum_nrj1.py           tka=data/todo.TKA</t>
+  </si>
+  <si>
+    <t>python3 spectrum_plot4.py         csv=$path_csv   case=todo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=todo  serv=1 </t>
+  </si>
+  <si>
+    <t>python3 spectrum_nrj1.py            tka=../irrad/petale/hpge_data/calib/Fu/2020_09_29_12_00_00_Fu_p13_Eu152-2020.TKA</t>
+  </si>
+  <si>
+    <t>python3 spectrum_nrj2.py            tka=test_data/spectro_files/calib_spectra/2020_09_29_12_00_00_Fu_p13_Eu152-2020.TKA</t>
+  </si>
+  <si>
+    <t>python3 spectrum_plot4.py         csv=$path_csv   case=Eu152_Fu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter11.py  csv=$path_csv   case=Eu152_Fu  serv=1 </t>
+  </si>
+  <si>
+    <t>python3 spectrum_plot4.py         csv=$path_csv   case=Eu152-2021_Fu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Eu152-2021_Fu  serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Co60_Fu   serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Mn54_Fu   serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Cs137_Fu    serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Cs134_Fu    serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Zn65_Fu     serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Co57_Fu    serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Na22_Fu   serv=1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">python3 spectrum_counter5.py  csv=$path_csv   case=Ba133_Fu    serv=1 </t>
+  </si>
+  <si>
+    <t>python3  check_cascade1.py</t>
+  </si>
+  <si>
+    <t>python3  spectrum_calib2.py   csv=$path_csv   case=Fu_p13_oct_2020</t>
   </si>
 </sst>
 </file>
@@ -832,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -849,9 +849,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1274,7 +1272,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1282,7 +1280,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
@@ -1394,7 +1392,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="B20" t="s">
         <v>30</v>
@@ -1407,7 +1405,7 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="B23" t="s">
         <v>32</v>
@@ -1451,7 +1449,7 @@
         <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
@@ -1461,35 +1459,35 @@
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="C36" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="C37" t="s">
-        <v>42</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
         <v>45</v>
-      </c>
-      <c r="B41" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -1498,128 +1496,128 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="K43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" t="s">
         <v>49</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>50</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>51</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>52</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>53</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>54</v>
       </c>
-      <c r="G44" t="s">
+      <c r="H44" t="s">
         <v>55</v>
       </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>56</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>57</v>
       </c>
-      <c r="J44" t="s">
+      <c r="K44" t="s">
         <v>58</v>
       </c>
-      <c r="K44" t="s">
+      <c r="L44" t="s">
         <v>59</v>
       </c>
-      <c r="L44" t="s">
+      <c r="M44" t="s">
         <v>60</v>
       </c>
-      <c r="M44" t="s">
+      <c r="N44" t="s">
+        <v>54</v>
+      </c>
+      <c r="O44" t="s">
         <v>61</v>
       </c>
-      <c r="N44" t="s">
-        <v>55</v>
-      </c>
-      <c r="O44" t="s">
+      <c r="P44" t="s">
         <v>62</v>
       </c>
-      <c r="P44" t="s">
+      <c r="Q44" t="s">
         <v>63</v>
-      </c>
-      <c r="Q44" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
+        <v>49</v>
+      </c>
+      <c r="C45" t="s">
         <v>50</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>51</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>52</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>53</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>54</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>55</v>
       </c>
-      <c r="H45" t="s">
+      <c r="I45" t="s">
         <v>56</v>
       </c>
-      <c r="I45" t="s">
-        <v>57</v>
-      </c>
       <c r="J45" t="s">
+        <v>64</v>
+      </c>
+      <c r="K45" t="s">
         <v>65</v>
       </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
         <v>66</v>
       </c>
-      <c r="L45" t="s">
+      <c r="M45" t="s">
         <v>67</v>
       </c>
-      <c r="M45" t="s">
-        <v>68</v>
-      </c>
       <c r="N45" t="s">
+        <v>54</v>
+      </c>
+      <c r="O45" t="s">
         <v>55</v>
       </c>
-      <c r="O45" t="s">
-        <v>56</v>
-      </c>
       <c r="P45" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q45" t="s">
         <v>63</v>
-      </c>
-      <c r="Q45" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="K46" t="s">
+        <v>68</v>
+      </c>
+      <c r="O46" t="s">
         <v>69</v>
-      </c>
-      <c r="O46" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="O47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -1630,103 +1628,103 @@
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
       <c r="K48" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C49" t="s">
         <v>50</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>51</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>52</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
         <v>53</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
+        <v>55</v>
+      </c>
+      <c r="H49" t="s">
+        <v>56</v>
+      </c>
+      <c r="I49" t="s">
+        <v>57</v>
+      </c>
+      <c r="J49" t="s">
+        <v>58</v>
+      </c>
+      <c r="K49" t="s">
+        <v>59</v>
+      </c>
+      <c r="L49" t="s">
+        <v>60</v>
+      </c>
+      <c r="M49" t="s">
         <v>54</v>
       </c>
-      <c r="G49" t="s">
-        <v>56</v>
-      </c>
-      <c r="H49" t="s">
-        <v>57</v>
-      </c>
-      <c r="I49" t="s">
-        <v>58</v>
-      </c>
-      <c r="J49" t="s">
-        <v>59</v>
-      </c>
-      <c r="K49" t="s">
-        <v>60</v>
-      </c>
-      <c r="L49" t="s">
+      <c r="N49" t="s">
         <v>61</v>
       </c>
-      <c r="M49" t="s">
-        <v>55</v>
-      </c>
-      <c r="N49" t="s">
-        <v>62</v>
-      </c>
       <c r="O49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50" t="s">
         <v>50</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>51</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>52</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>53</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
+        <v>55</v>
+      </c>
+      <c r="H50" t="s">
+        <v>56</v>
+      </c>
+      <c r="I50" t="s">
+        <v>57</v>
+      </c>
+      <c r="J50" t="s">
+        <v>58</v>
+      </c>
+      <c r="K50" t="s">
+        <v>59</v>
+      </c>
+      <c r="L50" t="s">
+        <v>60</v>
+      </c>
+      <c r="M50" t="s">
         <v>54</v>
       </c>
-      <c r="G50" t="s">
-        <v>56</v>
-      </c>
-      <c r="H50" t="s">
-        <v>57</v>
-      </c>
-      <c r="I50" t="s">
-        <v>58</v>
-      </c>
-      <c r="J50" t="s">
-        <v>59</v>
-      </c>
-      <c r="K50" t="s">
-        <v>60</v>
-      </c>
-      <c r="L50" t="s">
+      <c r="N50" t="s">
         <v>61</v>
       </c>
-      <c r="M50" t="s">
-        <v>55</v>
-      </c>
-      <c r="N50" t="s">
-        <v>62</v>
-      </c>
       <c r="O50" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -1734,359 +1732,359 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>75</v>
+      </c>
+      <c r="B54" t="s">
         <v>76</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>77</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>78</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>79</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>80</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>81</v>
       </c>
-      <c r="G54" t="s">
+      <c r="I54" t="s">
         <v>82</v>
-      </c>
-      <c r="I54" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
+        <v>83</v>
+      </c>
+      <c r="C55" t="s">
         <v>84</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>85</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>86</v>
-      </c>
-      <c r="E55" t="s">
-        <v>87</v>
       </c>
       <c r="F55">
         <v>0.5</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O55" s="4"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
+        <v>88</v>
+      </c>
+      <c r="C56" t="s">
+        <v>84</v>
+      </c>
+      <c r="D56" t="s">
+        <v>85</v>
+      </c>
+      <c r="E56" t="s">
         <v>89</v>
-      </c>
-      <c r="C56" t="s">
-        <v>85</v>
-      </c>
-      <c r="D56" t="s">
-        <v>86</v>
-      </c>
-      <c r="E56" t="s">
-        <v>90</v>
       </c>
       <c r="F56">
         <v>2</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O56" s="4"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
+        <v>91</v>
+      </c>
+      <c r="C57" t="s">
         <v>92</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>93</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>94</v>
-      </c>
-      <c r="E57" t="s">
-        <v>95</v>
       </c>
       <c r="F57">
         <v>0.52083333330000003</v>
       </c>
       <c r="G57" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I57" t="s">
         <v>96</v>
-      </c>
-      <c r="I57" t="s">
-        <v>97</v>
       </c>
       <c r="O57" s="4"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
+        <v>97</v>
+      </c>
+      <c r="C58" t="s">
         <v>98</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>99</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>100</v>
-      </c>
-      <c r="E58" t="s">
-        <v>101</v>
       </c>
       <c r="F58">
         <v>0.50274223029999998</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I58" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O58" s="4"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
+        <v>102</v>
+      </c>
+      <c r="C59" t="s">
         <v>103</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
         <v>104</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>105</v>
-      </c>
-      <c r="E59" t="s">
-        <v>106</v>
       </c>
       <c r="F59">
         <v>0.71428571429999999</v>
       </c>
       <c r="G59" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I59" t="s">
         <v>96</v>
-      </c>
-      <c r="I59" t="s">
-        <v>97</v>
       </c>
       <c r="O59" s="4"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" t="s">
         <v>107</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>108</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>109</v>
-      </c>
-      <c r="E60" t="s">
-        <v>110</v>
       </c>
       <c r="F60">
         <v>0.51424050629999996</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I60" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="O60" s="4"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
+        <v>111</v>
+      </c>
+      <c r="C61" t="s">
         <v>112</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
+        <v>108</v>
+      </c>
+      <c r="E61" t="s">
         <v>113</v>
-      </c>
-      <c r="D61" t="s">
-        <v>109</v>
-      </c>
-      <c r="E61" t="s">
-        <v>114</v>
       </c>
       <c r="F61">
         <v>0.51165434909999996</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I61" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O61" s="4"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
+        <v>115</v>
+      </c>
+      <c r="C62" t="s">
+        <v>84</v>
+      </c>
+      <c r="D62" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" t="s">
         <v>116</v>
-      </c>
-      <c r="C62" t="s">
-        <v>85</v>
-      </c>
-      <c r="D62" t="s">
-        <v>86</v>
-      </c>
-      <c r="E62" t="s">
-        <v>117</v>
       </c>
       <c r="F62">
         <v>0.83179297600000002</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O62" s="4"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C63" t="s">
+        <v>84</v>
+      </c>
+      <c r="D63" t="s">
         <v>85</v>
       </c>
-      <c r="D63" t="s">
-        <v>86</v>
-      </c>
       <c r="E63" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F63">
         <v>0.83179297600000002</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I63" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O63" s="4"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
+        <v>119</v>
+      </c>
+      <c r="C64" t="s">
         <v>120</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>121</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" t="s">
         <v>122</v>
-      </c>
-      <c r="E64" t="s">
-        <v>123</v>
       </c>
       <c r="F64">
         <v>0.56338028169999999</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I64" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O64" s="4"/>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
+        <v>124</v>
+      </c>
+      <c r="C65" t="s">
         <v>125</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>126</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>127</v>
-      </c>
-      <c r="E65" t="s">
-        <v>128</v>
       </c>
       <c r="F65">
         <v>0.50746268660000005</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I65" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O65" s="4"/>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
+        <v>129</v>
+      </c>
+      <c r="C66" t="s">
         <v>130</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>131</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>132</v>
-      </c>
-      <c r="E66" t="s">
-        <v>133</v>
       </c>
       <c r="F66">
         <v>0.55309734509999997</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I66" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O66" s="4"/>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C67" t="s">
+        <v>84</v>
+      </c>
+      <c r="D67" t="s">
         <v>85</v>
       </c>
-      <c r="D67" t="s">
-        <v>86</v>
-      </c>
       <c r="E67" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F67">
         <v>0.83179297600000002</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I67" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O67" s="4"/>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C68" t="s">
+        <v>84</v>
+      </c>
+      <c r="D68" t="s">
         <v>85</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>86</v>
-      </c>
-      <c r="E68" t="s">
-        <v>87</v>
       </c>
       <c r="F68">
         <v>0.5</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
@@ -2106,7 +2104,7 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2115,11 +2113,11 @@
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
       <c r="H72" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I72" s="3"/>
       <c r="J72" s="3" t="s">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="3"/>
@@ -2130,24 +2128,24 @@
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C73" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>143</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
       <c r="H73" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I73" s="3"/>
       <c r="J73" s="3" t="s">
-        <v>145</v>
+        <v>201</v>
       </c>
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
@@ -2158,10 +2156,10 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
@@ -2169,11 +2167,11 @@
       <c r="F74" s="3"/>
       <c r="G74" s="3"/>
       <c r="H74" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I74" s="3"/>
       <c r="J74" s="3" t="s">
-        <v>149</v>
+        <v>202</v>
       </c>
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
@@ -2184,10 +2182,10 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
@@ -2206,10 +2204,10 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C76" s="11">
         <v>0</v>
@@ -2222,7 +2220,7 @@
       </c>
       <c r="F76" s="11"/>
       <c r="G76" s="11" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
@@ -2236,19 +2234,19 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="13" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B80" s="13"/>
       <c r="C80" s="13"/>
       <c r="D80" s="13"/>
       <c r="E80" s="13"/>
       <c r="J80" t="s">
-        <v>155</v>
+        <v>203</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="13" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B81" s="13"/>
       <c r="C81" s="13"/>
@@ -2257,7 +2255,7 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="13" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B82" s="13"/>
       <c r="C82" s="13"/>
@@ -2266,55 +2264,55 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="G83" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G84" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="G85" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B86" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B87" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B88" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B89" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C89">
         <v>4.8492835847637004</v>
@@ -2325,50 +2323,50 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="G91" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="G92" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B93" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B94" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B95" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B96" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C96">
         <v>4.8492835847637004</v>
@@ -2379,47 +2377,47 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G98" t="s">
-        <v>167</v>
+        <v>209</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B99" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B100" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B101" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B102" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C102">
         <v>4.8492835847637004</v>
@@ -2430,47 +2428,47 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="G104" t="s">
-        <v>171</v>
+        <v>210</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B105" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B106" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B107" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B108" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C108">
         <v>4.8492835847637004</v>
@@ -2481,47 +2479,47 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="G110" t="s">
-        <v>175</v>
+        <v>211</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B111" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B112" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B113" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B114" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C114">
         <v>4.8492835847637004</v>
@@ -2532,50 +2530,50 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G116" t="s">
-        <v>179</v>
+        <v>212</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B117" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C117" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B118" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B119" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B120" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C120">
         <v>4.8492835847637004</v>
@@ -2586,47 +2584,47 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="G122" t="s">
-        <v>183</v>
+        <v>213</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B123" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B124" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B125" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B126" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C126">
         <v>4.8492835847637004</v>
@@ -2637,47 +2635,47 @@
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="G128" t="s">
-        <v>187</v>
+        <v>214</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B129" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B130" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B131" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B132" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C132">
         <v>4.8492835847637004</v>
@@ -2688,47 +2686,47 @@
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="G134" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B136" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B137" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B138" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C138">
         <v>4.8492835847637004</v>
@@ -2739,47 +2737,47 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="G140" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B141" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B142" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B143" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B144" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C144">
         <v>4.8492835847637004</v>
@@ -2790,20 +2788,20 @@
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="G148" s="2" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="B149">
         <v>7</v>
@@ -2812,12 +2810,12 @@
         <v>7</v>
       </c>
       <c r="G149" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="B150">
         <v>1</v>
@@ -2825,93 +2823,72 @@
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="B151" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="B152" t="s">
-        <v>206</v>
+        <v>190</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B159" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B160" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="161" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B161" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
     </row>
     <row r="162" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B162" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
     <row r="166" spans="2:7" x14ac:dyDescent="0.35">
       <c r="G166" s="2"/>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A183" s="16"/>
-      <c r="B183" s="16"/>
-      <c r="C183" s="16"/>
-      <c r="D183" s="16"/>
-      <c r="E183" s="16"/>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A184" s="16"/>
-      <c r="B184" s="16"/>
-      <c r="C184" s="16"/>
-      <c r="D184" s="16"/>
-      <c r="E184" s="16"/>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A185" s="16"/>
-      <c r="B185" s="16"/>
-      <c r="C185" s="16"/>
-      <c r="D185" s="16"/>
-      <c r="E185" s="16"/>
     </row>
     <row r="198" spans="7:7" x14ac:dyDescent="0.35">
       <c r="G198" s="2"/>
@@ -2926,387 +2903,289 @@
     <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="G223" s="2"/>
     </row>
-    <row r="254" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="255" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="256" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="257" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="258" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="259" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="260" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="261" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="262" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="263" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="264" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="265" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="266" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="267" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="268" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="269" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="E269" s="17"/>
-      <c r="F269" s="17"/>
-    </row>
-    <row r="270" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="E270" s="17"/>
-      <c r="F270" s="17"/>
-    </row>
-    <row r="271" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="E271" s="17"/>
-      <c r="F271" s="17"/>
-    </row>
-    <row r="272" spans="5:6" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="E272" s="17"/>
-      <c r="F272" s="17"/>
-    </row>
-    <row r="273" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="274" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="275" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="276" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="277" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="278" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="279" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="280" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="281" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="282" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="283" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="284" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="285" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="286" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="287" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="288" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C288" s="17"/>
-      <c r="D288" s="17"/>
-    </row>
-    <row r="289" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="290" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="291" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="292" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="293" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="294" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C294" s="17"/>
-      <c r="D294" s="17"/>
-    </row>
-    <row r="295" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="296" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="297" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="298" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="299" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="300" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="301" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="302" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="303" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="304" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="305" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="306" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="307" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="308" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C308" s="18"/>
-      <c r="D308" s="18"/>
-    </row>
-    <row r="309" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="310" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C310" s="18"/>
-    </row>
-    <row r="311" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="312" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="313" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="314" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="315" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="316" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="317" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C317" s="18"/>
-      <c r="D317" s="18"/>
-    </row>
-    <row r="318" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="319" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="320" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="321" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="322" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="323" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="324" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="325" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="326" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C326" s="18"/>
-      <c r="D326" s="18"/>
-    </row>
-    <row r="327" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="328" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="329" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="330" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="331" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="332" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="333" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="334" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="335" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C335" s="18"/>
-      <c r="D335" s="18"/>
-    </row>
-    <row r="336" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="337" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="338" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="339" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="340" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="341" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="342" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="343" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="344" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C344" s="18"/>
-      <c r="D344" s="18"/>
-    </row>
-    <row r="345" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="346" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="347" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="348" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="349" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="350" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="351" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="352" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="353" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="354" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="355" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C355" s="18"/>
-      <c r="D355" s="18"/>
-    </row>
-    <row r="356" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="357" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="358" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="359" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="360" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="361" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="362" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="363" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="364" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="365" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C365" s="18"/>
-      <c r="D365" s="18"/>
-    </row>
-    <row r="366" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="367" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="368" spans="3:4" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="369" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="370" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="371" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="372" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="373" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="374" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="375" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="376" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="377" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="378" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="379" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="380" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="381" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="382" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="383" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="384" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="385" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="386" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="387" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="388" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="389" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="390" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="391" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="392" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="393" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="394" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="395" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="396" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="397" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="398" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="399" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="400" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="401" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="402" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="403" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="404" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="405" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="406" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="407" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="408" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="409" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="410" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="411" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="412" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="413" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="414" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="415" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="416" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="417" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="418" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="419" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="420" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="421" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="422" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="423" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="424" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="425" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="426" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="427" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="428" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="429" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="430" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="431" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="432" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="433" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="434" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="435" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="436" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="437" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="438" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="439" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="440" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="441" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="442" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="443" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="444" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="445" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="446" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="447" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="448" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="449" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="450" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="451" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="452" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="453" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="454" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="455" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="456" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="457" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="458" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="459" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="460" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="461" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="462" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="463" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="464" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="465" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="466" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="467" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="468" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="469" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="470" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="471" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="472" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="473" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="474" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="475" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="476" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="477" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="478" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="479" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="480" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="481" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="482" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="483" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="484" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="485" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="486" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="487" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="488" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="489" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="490" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="491" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="492" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="493" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="494" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="495" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="496" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="497" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="498" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="499" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="500" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="501" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="502" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="503" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="504" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="505" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="506" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="507" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="508" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="509" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="510" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="511" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="512" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="513" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="514" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="515" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="516" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="517" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="518" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="519" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="520" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="521" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="522" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="523" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="524" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="525" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="526" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="527" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="528" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="529" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="530" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="531" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="532" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="533" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="534" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="535" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="536" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="537" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="538" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="539" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="540" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="541" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="542" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="543" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="544" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="545" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="546" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="547" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="548" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="549" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="550" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="551" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="552" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="553" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="554" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="555" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="556" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="557" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="558" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="559" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="560" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="561" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="562" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="563" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="564" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="565" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="566" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="567" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="568" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="569" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="570" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="571" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="572" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="573" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="574" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="575" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="576" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="577" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="578" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="579" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="580" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="581" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="582" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="583" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="584" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="585" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="586" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="587" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="588" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="589" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="590" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="591" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="592" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="593" s="16" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="254" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="255" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="256" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="269" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E269" s="16"/>
+      <c r="F269" s="16"/>
+    </row>
+    <row r="270" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E270" s="16"/>
+      <c r="F270" s="16"/>
+    </row>
+    <row r="271" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E271" s="16"/>
+      <c r="F271" s="16"/>
+    </row>
+    <row r="272" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E272" s="16"/>
+      <c r="F272" s="16"/>
+    </row>
+    <row r="288" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C288" s="16"/>
+      <c r="D288" s="16"/>
+    </row>
+    <row r="294" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C294" s="16"/>
+      <c r="D294" s="16"/>
+    </row>
+    <row r="308" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C308" s="14"/>
+      <c r="D308" s="14"/>
+    </row>
+    <row r="310" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C310" s="14"/>
+    </row>
+    <row r="317" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C317" s="14"/>
+      <c r="D317" s="14"/>
+    </row>
+    <row r="326" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C326" s="14"/>
+      <c r="D326" s="14"/>
+    </row>
+    <row r="335" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C335" s="14"/>
+      <c r="D335" s="14"/>
+    </row>
+    <row r="344" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C344" s="14"/>
+      <c r="D344" s="14"/>
+    </row>
+    <row r="355" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C355" s="14"/>
+      <c r="D355" s="14"/>
+    </row>
+    <row r="365" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C365" s="14"/>
+      <c r="D365" s="14"/>
+    </row>
+    <row r="369" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="370" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="371" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="372" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="373" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="374" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="375" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="376" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="377" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="378" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="379" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="380" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="381" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="382" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="383" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="384" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="385" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="386" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="387" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="388" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="389" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="390" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="391" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="392" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="393" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="394" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="395" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="396" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="397" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="398" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="399" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="400" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="401" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="402" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="403" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="404" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="405" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="406" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="407" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="408" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="409" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="410" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="411" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="412" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="413" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="414" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="415" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="416" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="417" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="418" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="419" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="420" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="421" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="422" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="423" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="424" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="425" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="426" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="427" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="428" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="429" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="430" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="431" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="432" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="433" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="434" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="435" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="436" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="437" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="438" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="439" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="440" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="441" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="442" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="443" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="444" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="445" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="446" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="447" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="448" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="449" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="450" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="451" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="452" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="453" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="454" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="455" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="456" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="457" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="458" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="459" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="460" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="461" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="462" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="463" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="464" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="465" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="466" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="467" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="468" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="469" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="470" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="471" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="472" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="473" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="474" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="475" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="476" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="477" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="478" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="479" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="480" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="481" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="482" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="483" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="484" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="485" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="486" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="487" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="488" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="489" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="490" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="491" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="492" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="493" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="494" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="495" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="496" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="497" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="498" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="499" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="500" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="501" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="502" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="503" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="504" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="505" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="506" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="507" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="508" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="509" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="510" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="511" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="512" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="513" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="514" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="515" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="516" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="517" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="518" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="519" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="520" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="521" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="522" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="523" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="524" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="525" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="526" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="527" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="528" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="529" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="530" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="531" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="532" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="533" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="534" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="535" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="536" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="537" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="538" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="539" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="540" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="541" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="542" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="543" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="544" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="545" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="546" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="547" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="548" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="549" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="550" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="551" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="552" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="553" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="554" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="555" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="556" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="557" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="558" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="559" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="560" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="561" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="562" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="563" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="564" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="565" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="566" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="567" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="568" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="569" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="570" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="571" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="572" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="573" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="574" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="575" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="576" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="577" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="578" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="579" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="580" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="581" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="582" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="583" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="584" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="585" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="586" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="587" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="588" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="589" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="590" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="591" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="592" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="593" customFormat="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>